<commit_message>
O-D takip kurallari revize edildi: StateMemory v1'e geri donuldu, Reporting modulu iyilestirildi.
</commit_message>
<xml_diff>
--- a/trafik_raporu_yogunburc.xlsx
+++ b/trafik_raporu_yogunburc.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -475,16 +475,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-10 10:43:01</t>
+          <t>2026-04-10 12:31:03</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>25 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>26 idli Otomobil 4 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -493,33 +493,33 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2 → 1 → 6</t>
+          <t>4 → 2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-10 10:43:05</t>
+          <t>2026-04-10 12:31:04</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>27 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>29 idli Otomobil 3 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -528,33 +528,33 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2 → 1 → 6</t>
+          <t>3 → 2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-10 10:43:07</t>
+          <t>2026-04-10 12:31:06</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>36 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>47 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -568,28 +568,28 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2 → 6</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-10 10:43:11</t>
+          <t>2026-04-10 12:31:07</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>28 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>49 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -603,28 +603,28 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2 → 1 → 6</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-10 10:43:17</t>
+          <t>2026-04-10 12:31:08</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>40 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>50 idli Otomobil 2 ten girdi 4 ten cikti</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -638,63 +638,63 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2 → 1 → 6</t>
+          <t>2 → 4</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-10 10:43:20</t>
+          <t>2026-04-10 12:31:13</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>83 idli Panelvan 1 ten girdi 4 ten cikti</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Otomobil</t>
+          <t>Panelvan</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2 → 1 → 6</t>
+          <t>1 → 4</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-10 10:43:21</t>
+          <t>2026-04-10 12:31:14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>46 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>87 idli Otomobil 1 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -703,33 +703,33 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2 → 6</t>
+          <t>1 → 4 → 2</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-10 10:43:25</t>
+          <t>2026-04-10 12:31:18</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>44 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>89 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>44</v>
+        <v>89</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -743,32 +743,32 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2 → 1 → 6</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-10 10:43:28</t>
+          <t>2026-04-10 12:31:19</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>42 idli Otobus 2 ten girdi 6 ten cikti</t>
+          <t>92 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Otobus</t>
+          <t>Otomobil</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -778,28 +778,28 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2 → 1 → 6</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-10 10:43:53</t>
+          <t>2026-04-10 12:31:19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>33 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>94 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>33</v>
+        <v>94</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -813,28 +813,28 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2 → 1 → 6</t>
+          <t>2 → 1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-10 10:44:04</t>
+          <t>2026-04-10 12:31:22</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>34 idli Otomobil 3 ten girdi 6 ten cikti</t>
+          <t>97 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -843,33 +843,33 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>3 → 2 → 1 → 6</t>
+          <t>2 → 1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-10 10:44:07</t>
+          <t>2026-04-10 12:31:24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>30 idli Otomobil 3 ten girdi 6 ten cikti</t>
+          <t>100 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -878,33 +878,33 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3 → 2 → 6</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-10 10:44:12</t>
+          <t>2026-04-10 12:31:24</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>37 idli Otomobil 3 ten girdi 6 ten cikti</t>
+          <t>101 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>37</v>
+        <v>101</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -913,33 +913,33 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3 → 2 → 6</t>
+          <t>2 → 1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-10 10:44:17</t>
+          <t>2026-04-10 12:31:25</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>63 idli Otomobil 3 ten girdi 6 ten cikti</t>
+          <t>99 idli Otomobil 4 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -948,33 +948,33 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3 → 2 → 1 → 6</t>
+          <t>4 → 1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-10 10:44:21</t>
+          <t>2026-04-10 12:31:26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>49 idli Otomobil 3 ten girdi 6 ten cikti</t>
+          <t>105 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>49</v>
+        <v>105</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -983,33 +983,33 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3 → 2 → 6</t>
+          <t>2 → 1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-10 10:44:22</t>
+          <t>2026-04-10 12:31:27</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>68 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>111 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>68</v>
+        <v>111</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1023,28 +1023,28 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2 → 1 → 6</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-10 10:44:26</t>
+          <t>2026-04-10 12:31:27</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>61 idli Otomobil 3 ten girdi 6 ten cikti</t>
+          <t>115 idli Otomobil 2 ten girdi 4 ten cikti</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1053,33 +1053,33 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>3 → 2 → 1 → 6</t>
+          <t>2 → 4</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-10 10:44:40</t>
+          <t>2026-04-10 12:31:28</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>72 idli Otomobil 3 ten girdi 6 ten cikti</t>
+          <t>117 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>72</v>
+        <v>117</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1088,33 +1088,33 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>3 → 2 → 6</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-10 10:44:51</t>
+          <t>2026-04-10 12:31:29</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>76 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>118 idli Otomobil 1 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>76</v>
+        <v>118</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1123,33 +1123,33 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>1 → 4 → 2</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-10 10:44:53</t>
+          <t>2026-04-10 12:31:29</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>79 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>122 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>79</v>
+        <v>122</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1158,33 +1158,33 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-10 10:44:55</t>
+          <t>2026-04-10 12:31:29</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>67 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>121 idli Otomobil 1 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>67</v>
+        <v>121</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1193,33 +1193,33 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>1 → 2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:03</t>
+          <t>2026-04-10 12:31:30</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>80 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>103 idli Otomobil 3 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1228,33 +1228,33 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>3 → 2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:10</t>
+          <t>2026-04-10 12:31:32</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>84 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>126 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>84</v>
+        <v>126</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1263,33 +1263,33 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:18</t>
+          <t>2026-04-10 12:31:33</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>85 idli Otomobil 3 ten girdi 6 ten cikti</t>
+          <t>119 idli Otomobil 3 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>85</v>
+        <v>119</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1303,63 +1303,63 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>3 → 2 → 1 → 6</t>
+          <t>3 → 2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:21</t>
+          <t>2026-04-10 12:31:34</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>94 idli Panelvan 5 ten girdi 3 ten cikti</t>
+          <t>132 idli Otomobil 1 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Panelvan</t>
+          <t>Otomobil</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>1 → 2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:33</t>
+          <t>2026-04-10 12:31:35</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>102 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>129 idli Otomobil 1 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>102</v>
+        <v>129</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1368,33 +1368,33 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>1 → 2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:34</t>
+          <t>2026-04-10 12:31:35</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>97 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>114 idli Otomobil 3 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1403,33 +1403,33 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>3 → 2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:34</t>
+          <t>2026-04-10 12:31:36</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>100 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>134 idli Otomobil 1 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>100</v>
+        <v>134</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1438,33 +1438,33 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>1 → 2</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:43</t>
+          <t>2026-04-10 12:31:37</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>107 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>135 idli Otomobil 1 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>107</v>
+        <v>135</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1473,33 +1473,33 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>1 → 4 → 2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:45</t>
+          <t>2026-04-10 12:31:37</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>110 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>146 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>110</v>
+        <v>146</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1508,33 +1508,33 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:45</t>
+          <t>2026-04-10 12:31:37</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>105 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>149 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>105</v>
+        <v>149</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1543,33 +1543,33 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:49</t>
+          <t>2026-04-10 12:31:37</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>83 idli Otomobil 2 ten girdi 1 ten cikti</t>
+          <t>147 idli Otomobil 1 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>83</v>
+        <v>147</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1578,33 +1578,33 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2 → 1</t>
+          <t>1 → 2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:49</t>
+          <t>2026-04-10 12:31:39</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>62 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>140 idli Otomobil 1 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>62</v>
+        <v>140</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1613,33 +1613,33 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2 → 1 → 6</t>
+          <t>1 → 2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:53</t>
+          <t>2026-04-10 12:31:39</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>114 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>151 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>114</v>
+        <v>151</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1648,33 +1648,33 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:53</t>
+          <t>2026-04-10 12:31:40</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>117 idli Otomobil 5 ten girdi 3 ten cikti</t>
+          <t>150 idli Otomobil 1 ten girdi 2 ten cikti</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>117</v>
+        <v>150</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1683,33 +1683,33 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>5 → 3</t>
+          <t>1 → 4 → 2</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-10 10:45:54</t>
+          <t>2026-04-10 12:31:40</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>48 idli Otomobil 2 ten girdi 6 ten cikti</t>
+          <t>156 idli Otomobil 2 ten girdi 1 ten cikti</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>48</v>
+        <v>156</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1723,82 +1723,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2 → 1 → 6</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2026-04-10 10:45:58</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>131 idli Otomobil 5 ten girdi 3 ten cikti</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>131</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Otomobil</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>5 → 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2026-04-10 10:45:58</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>56 idli Otomobil 2 ten girdi 6 ten cikti</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>56</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Otomobil</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2 → 6</t>
+          <t>2 → 3 → 1</t>
         </is>
       </c>
     </row>

</xml_diff>